<commit_message>
modified results ouput to include images
</commit_message>
<xml_diff>
--- a/outputs/results/recordings_summary.xlsx
+++ b/outputs/results/recordings_summary.xlsx
@@ -9,6 +9,7 @@
   <sheets>
     <sheet name="Overview" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Recording 1" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Recording 2" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -172,6 +173,86 @@
       </nvPicPr>
       <blipFill>
         <a:blip cstate="print" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>7</col>
+      <colOff>0</colOff>
+      <row>30</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5897879" cy="4411980"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="2" name="Image 2" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>7</col>
+      <colOff>0</colOff>
+      <row>0</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="11430000" cy="5715000"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>7</col>
+      <colOff>0</colOff>
+      <row>30</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5897879" cy="4411980"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="2" name="Image 2" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId2"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -488,7 +569,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F8"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -526,155 +607,136 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>alive 1</t>
+          <t>alive</t>
         </is>
       </c>
       <c r="B2" t="n">
         <v>1</v>
       </c>
       <c r="C2" t="n">
-        <v>3</v>
+        <v>21</v>
       </c>
       <c r="D2" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="E2" t="n">
-        <v>3</v>
+        <v>16</v>
       </c>
       <c r="F2" t="n">
-        <v>0</v>
+        <v>23.81</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>dead 1</t>
+          <t>dead</t>
         </is>
       </c>
       <c r="B3" t="n">
         <v>1</v>
       </c>
       <c r="C3" t="n">
-        <v>3</v>
+        <v>35</v>
       </c>
       <c r="D3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E3" t="n">
+        <v>35</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Zone ID</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>recording</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Total Mites</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Alive Mites</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Dead Mites</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Survival %</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>alive</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
         <v>2</v>
       </c>
+      <c r="C2" t="n">
+        <v>21</v>
+      </c>
+      <c r="D2" t="n">
+        <v>5</v>
+      </c>
+      <c r="E2" t="n">
+        <v>16</v>
+      </c>
+      <c r="F2" t="n">
+        <v>23.81</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>2</v>
+      </c>
+      <c r="C3" t="n">
+        <v>35</v>
+      </c>
+      <c r="D3" t="n">
+        <v>0</v>
+      </c>
       <c r="E3" t="n">
-        <v>1</v>
+        <v>35</v>
       </c>
       <c r="F3" t="n">
-        <v>66.67</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>test 1</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
-        <v>1</v>
-      </c>
-      <c r="C4" t="n">
-        <v>4</v>
-      </c>
-      <c r="D4" t="n">
         <v>0</v>
-      </c>
-      <c r="E4" t="n">
-        <v>4</v>
-      </c>
-      <c r="F4" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>test 2</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>1</v>
-      </c>
-      <c r="C5" t="n">
-        <v>6</v>
-      </c>
-      <c r="D5" t="n">
-        <v>1</v>
-      </c>
-      <c r="E5" t="n">
-        <v>5</v>
-      </c>
-      <c r="F5" t="n">
-        <v>16.67</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>untreated</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
-        <v>1</v>
-      </c>
-      <c r="C6" t="n">
-        <v>9</v>
-      </c>
-      <c r="D6" t="n">
-        <v>3</v>
-      </c>
-      <c r="E6" t="n">
-        <v>6</v>
-      </c>
-      <c r="F6" t="n">
-        <v>33.33</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>venom 1</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
-        <v>1</v>
-      </c>
-      <c r="C7" t="n">
-        <v>5</v>
-      </c>
-      <c r="D7" t="n">
-        <v>2</v>
-      </c>
-      <c r="E7" t="n">
-        <v>3</v>
-      </c>
-      <c r="F7" t="n">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>venom 2</t>
-        </is>
-      </c>
-      <c r="B8" t="n">
-        <v>1</v>
-      </c>
-      <c r="C8" t="n">
-        <v>5</v>
-      </c>
-      <c r="D8" t="n">
-        <v>1</v>
-      </c>
-      <c r="E8" t="n">
-        <v>4</v>
-      </c>
-      <c r="F8" t="n">
-        <v>20</v>
       </c>
     </row>
   </sheetData>

</xml_diff>